<commit_message>
docs(tutorials): FEM-2 runs LEM-8's model as published — 4 ft at both ends
Same model, two engines: Spencer 1.587; SSRM 1.559 elastic-perfectly-
plastic and 1.512 with the residual, identical from a 3,000 budget. At
the published ramps the two limits show in one field — four lines at
their bond limit at the buried tips, one at its rupture limit mid-bar —
which is the reading exercise. The overburden law now moves both
engines (1.559 -> 1.543, 1.587 -> 1.559).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_reinforced_slope.xlsx
+++ b/docs/tutorials/files/xslope_reinforced_slope.xlsx
@@ -3346,7 +3346,7 @@
         <v>4.0</v>
       </c>
       <c r="L3" s="3">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
@@ -3419,7 +3419,7 @@
         <v>4.0</v>
       </c>
       <c r="L4" s="3">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
@@ -3486,7 +3486,7 @@
         <v>4.0</v>
       </c>
       <c r="L5" s="3">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
@@ -3553,7 +3553,7 @@
         <v>4.0</v>
       </c>
       <c r="L6" s="3">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
@@ -3617,7 +3617,7 @@
         <v>4.0</v>
       </c>
       <c r="L7" s="3">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
@@ -3681,7 +3681,7 @@
         <v>4.0</v>
       </c>
       <c r="L8" s="3">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>

</xml_diff>